<commit_message>
fix(inspeccion): corregir referencia de seccion en Anexo A (5.3 -> 5.5, matriz de trazabilidad)
</commit_message>
<xml_diff>
--- a/02_Inspeccion/AnexoA_checklists/AnexoA_checklist_Moderador_Lector_Andy_Mendoza.xlsx
+++ b/02_Inspeccion/AnexoA_checklists/AnexoA_checklist_Moderador_Lector_Andy_Mendoza.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andy Mendoza\Desktop\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F393B1A-7537-41B7-9272-6DDFC7CBCA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97D2E31E-A65F-4191-B2A6-FFED8ECF0588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -100,15 +100,9 @@
     <t>¿Todos los atributos exigidos por la plantilla (entradas, salidas, precondiciones, postcondiciones, prioridad, criterio de verificación) están presentes y no vacíos?</t>
   </si>
   <si>
-    <t>Sección 5.1 vs. Sección 5.3</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
-    <t>La clasificación de requisitos (5.1) declara 59 requisitos vigentes (25 RF + 16 RNF + 9 RD + 9 RL), pero la matriz de trazabilidad (5.3) declara cubrir "los 50 elementos especificados", que corresponde solo a RF+RNF+RD, sin incluir los 9 requisitos legales (RL) ni explicar por qué quedan fuera de la matriz.</t>
-  </si>
-  <si>
     <t>RF-01</t>
   </si>
   <si>
@@ -127,9 +121,6 @@
     <t>La definición de "titular" en la Sección 2 establece que el historial médico de la mascota no constituye, en sí mismo, un dato personal protegido. Sin embargo, RL-07 afirma que "el historial clínico de la mascota se protege como extensión indirecta de esos datos". Ambas afirmaciones generan una contradicción sobre si el historial médico está o no protegido como dato personal.</t>
   </si>
   <si>
-    <t>Sección 5.3, matriz de trazabilidad</t>
-  </si>
-  <si>
     <t>El texto indica que "la matriz completa, con sus 40 filas (TR-01 a TR-40), se presenta en el Apéndice D", pero dos oraciones después declara que "la matriz cubre los 50 elementos especificados" y "de las 50 filas...". Existe una inconsistencia numérica entre 40 y 50 filas/elementos dentro del mismo párrafo.</t>
   </si>
   <si>
@@ -176,6 +167,15 @@
   </si>
   <si>
     <t>08/08/2026 — 11:15</t>
+  </si>
+  <si>
+    <t>Sección 5.5, matriz de trazabilidad</t>
+  </si>
+  <si>
+    <t>La clasificación de requisitos (5.1) declara 59 requisitos vigentes (25 RF + 16 RNF + 9 RD + 9 RL), pero la matriz de trazabilidad (5.5) declara cubrir "los 50 elementos especificados", que corresponde solo a RF+RNF+RD, sin incluir los 9 requisitos legales (RL) ni explicar por qué quedan fuera de la matriz.</t>
+  </si>
+  <si>
+    <t>Sección 5.1 vs. Sección 5.5</t>
   </si>
 </sst>
 </file>
@@ -293,13 +293,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -309,36 +327,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -729,24 +728,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -787,7 +786,7 @@
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -795,7 +794,7 @@
         <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -804,14 +803,14 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
@@ -834,232 +833,232 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="13">
+      <c r="A11" s="4">
         <v>1</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="13">
+      <c r="A12" s="4">
         <v>2</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
     </row>
     <row r="13" spans="1:6" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="13">
+      <c r="A13" s="4">
         <v>3</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="F13" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <v>4</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="E14" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="13">
-        <v>4</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16" t="s">
+    <row r="15" spans="1:6" ht="115.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="4">
+        <v>5</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="17" t="s">
+      <c r="C15" s="6" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="115.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="13">
-        <v>5</v>
-      </c>
-      <c r="B15" s="14" t="s">
+      <c r="D15" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="E15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="16" t="s">
+    </row>
+    <row r="16" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
+        <v>6</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="6"/>
+      <c r="D16" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="F15" s="17" t="s">
+    </row>
+    <row r="17" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="A17" s="4">
+        <v>7</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="13">
-        <v>6</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16" t="s">
+      <c r="C17" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="F16" s="17" t="s">
+      <c r="D17" s="7" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A17" s="13">
-        <v>7</v>
-      </c>
-      <c r="B17" s="14" t="s">
+      <c r="E17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="15" t="s">
+    </row>
+    <row r="18" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="4">
+        <v>8</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="6"/>
+      <c r="D18" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="E18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" s="17" t="s">
+    </row>
+    <row r="19" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4">
+        <v>9</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="13">
-        <v>8</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16" t="s">
+      <c r="C19" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18" s="17" t="s">
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4">
+        <v>10</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4">
+        <v>11</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="13">
-        <v>9</v>
-      </c>
-      <c r="B19" s="14" t="s">
+      <c r="C21" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+    </row>
+    <row r="22" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="4">
+        <v>12</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="10"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-    </row>
-    <row r="20" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="13">
-        <v>10</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-    </row>
-    <row r="21" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="13">
-        <v>11</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-    </row>
-    <row r="22" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="13">
-        <v>12</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="4"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="18">
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="9">
         <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
+        <v>45</v>
+      </c>
+      <c r="B27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" s="19">
+        <v>46</v>
+      </c>
+      <c r="B28" s="15">
         <v>46242</v>
       </c>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>